<commit_message>
Complete MAP data regression analysis project
</commit_message>
<xml_diff>
--- a/data/2022_2023 MAP Data.xlsx
+++ b/data/2022_2023 MAP Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\map-regression\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7108260C-9C6B-4FAD-912E-683EB66A8DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE86E4C5-811C-4BF6-A462-1050101FB5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22180" windowHeight="14860" xr2:uid="{449B78BD-E0C3-49C0-8A5B-B657B24BCA65}"/>
+    <workbookView xWindow="360" yWindow="1040" windowWidth="21600" windowHeight="11720" xr2:uid="{449B78BD-E0C3-49C0-8A5B-B657B24BCA65}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
     <t>Geometry</t>
   </si>
   <si>
-    <t>Rit Score</t>
+    <t>RitScore</t>
   </si>
 </sst>
 </file>
@@ -89,10 +89,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -432,900 +431,899 @@
   <dimension ref="A1:B112"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" style="1"/>
+    <col min="1" max="1" width="8.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
         <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
         <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="2">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1">
         <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="2">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="1">
         <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="2">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1">
         <v>236</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="1">
         <v>233</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="2">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="1">
         <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" s="2">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1">
         <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="2">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="1">
         <v>228</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="2">
+      <c r="A11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="1">
         <v>239</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B12" s="2">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="1">
         <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" s="2">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="1">
         <v>233</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14" s="2">
+      <c r="A14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1">
         <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B15" s="2">
+      <c r="A15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" s="1">
         <v>228</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B16" s="2">
+      <c r="A16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1">
         <v>229</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17" s="2">
+      <c r="A17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1">
         <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B18" s="2">
+      <c r="A18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1">
         <v>211</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B19" s="2">
+      <c r="A19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B19" s="1">
         <v>230</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B20" s="2">
+      <c r="A20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="1">
         <v>229</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B21" s="2">
+      <c r="A21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="1">
         <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" s="2">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1">
         <v>231</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="2">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="1">
         <v>239</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B24" s="2">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="1">
         <v>234</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B25" s="2">
+      <c r="A25" t="s">
+        <v>1</v>
+      </c>
+      <c r="B25" s="1">
         <v>251</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="2">
+      <c r="A26" t="s">
+        <v>1</v>
+      </c>
+      <c r="B26" s="1">
         <v>261</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B27" s="2">
+      <c r="A27" t="s">
+        <v>1</v>
+      </c>
+      <c r="B27" s="1">
         <v>251</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B28" s="2">
+      <c r="A28" t="s">
+        <v>1</v>
+      </c>
+      <c r="B28" s="1">
         <v>244</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="2">
+      <c r="A29" t="s">
+        <v>1</v>
+      </c>
+      <c r="B29" s="1">
         <v>231</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B30" s="2">
+      <c r="A30" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" s="1">
         <v>251</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B31" s="2">
+      <c r="A31" t="s">
+        <v>1</v>
+      </c>
+      <c r="B31" s="1">
         <v>258</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B32" s="2">
+      <c r="A32" t="s">
+        <v>1</v>
+      </c>
+      <c r="B32" s="1">
         <v>247</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B33" s="2">
+      <c r="A33" t="s">
+        <v>1</v>
+      </c>
+      <c r="B33" s="1">
         <v>263</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B34" s="2">
+      <c r="A34" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="1">
         <v>241</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B35" s="2">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="1">
         <v>253</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B36" s="2">
+      <c r="A36" t="s">
+        <v>1</v>
+      </c>
+      <c r="B36" s="1">
         <v>254</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="2">
+      <c r="A37" t="s">
+        <v>1</v>
+      </c>
+      <c r="B37" s="1">
         <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B38" s="2">
+      <c r="A38" t="s">
+        <v>1</v>
+      </c>
+      <c r="B38" s="1">
         <v>252</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B39" s="2">
+      <c r="A39" t="s">
+        <v>1</v>
+      </c>
+      <c r="B39" s="1">
         <v>245</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B40" s="2">
+      <c r="A40" t="s">
+        <v>1</v>
+      </c>
+      <c r="B40" s="1">
         <v>263</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B41" s="2">
+      <c r="A41" t="s">
+        <v>1</v>
+      </c>
+      <c r="B41" s="1">
         <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B42" s="2">
+      <c r="A42" t="s">
+        <v>1</v>
+      </c>
+      <c r="B42" s="1">
         <v>240</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B43" s="2">
+      <c r="A43" t="s">
+        <v>1</v>
+      </c>
+      <c r="B43" s="1">
         <v>249</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B44" s="2">
+      <c r="A44" t="s">
+        <v>1</v>
+      </c>
+      <c r="B44" s="1">
         <v>260</v>
       </c>
     </row>
-    <row r="45" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B45" s="2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>1</v>
+      </c>
+      <c r="B45" s="1">
         <v>252</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B46" s="2">
+      <c r="A46" t="s">
+        <v>1</v>
+      </c>
+      <c r="B46" s="1">
         <v>247</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B47" s="2">
+      <c r="A47" t="s">
+        <v>1</v>
+      </c>
+      <c r="B47" s="1">
         <v>245</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B48" s="2">
+      <c r="A48" t="s">
+        <v>1</v>
+      </c>
+      <c r="B48" s="1">
         <v>247</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B49" s="2">
+      <c r="A49" t="s">
+        <v>1</v>
+      </c>
+      <c r="B49" s="1">
         <v>245</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B50" s="2">
+      <c r="A50" t="s">
+        <v>1</v>
+      </c>
+      <c r="B50" s="1">
         <v>257</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B51" s="2">
+      <c r="A51" t="s">
+        <v>1</v>
+      </c>
+      <c r="B51" s="1">
         <v>246</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A52" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B52" s="2">
+      <c r="A52" t="s">
+        <v>1</v>
+      </c>
+      <c r="B52" s="1">
         <v>240</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A53" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B53" s="2">
+      <c r="A53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B53" s="1">
         <v>246</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B54" s="2">
+      <c r="A54" t="s">
+        <v>1</v>
+      </c>
+      <c r="B54" s="1">
         <v>252</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B55" s="2">
+      <c r="A55" t="s">
+        <v>1</v>
+      </c>
+      <c r="B55" s="1">
         <v>241</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A56" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B56" s="2">
+      <c r="A56" t="s">
+        <v>1</v>
+      </c>
+      <c r="B56" s="1">
         <v>261</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A57" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B57" s="2">
+      <c r="A57" t="s">
+        <v>1</v>
+      </c>
+      <c r="B57" s="1">
         <v>248</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A58" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B58" s="2">
+      <c r="A58" t="s">
+        <v>1</v>
+      </c>
+      <c r="B58" s="1">
         <v>250</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A59" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B59" s="2">
+      <c r="A59" t="s">
+        <v>1</v>
+      </c>
+      <c r="B59" s="1">
         <v>243</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A60" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B60" s="2">
+      <c r="A60" t="s">
+        <v>1</v>
+      </c>
+      <c r="B60" s="1">
         <v>247</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A61" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B61" s="2">
+      <c r="A61" t="s">
+        <v>1</v>
+      </c>
+      <c r="B61" s="1">
         <v>261</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A62" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B62" s="2">
+      <c r="A62" t="s">
+        <v>1</v>
+      </c>
+      <c r="B62" s="1">
         <v>237</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A63" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B63" s="2">
+      <c r="A63" t="s">
+        <v>1</v>
+      </c>
+      <c r="B63" s="1">
         <v>250</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A64" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B64" s="2">
+      <c r="A64" t="s">
+        <v>0</v>
+      </c>
+      <c r="B64" s="1">
         <v>231</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A65" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B65" s="2">
+      <c r="A65" t="s">
+        <v>0</v>
+      </c>
+      <c r="B65" s="1">
         <v>237</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A66" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B66" s="2">
+      <c r="A66" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="1">
         <v>238</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A67" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B67" s="2">
+      <c r="A67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B67" s="1">
         <v>253</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A68" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" s="2">
+      <c r="A68" t="s">
+        <v>0</v>
+      </c>
+      <c r="B68" s="1">
         <v>240</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A69" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B69" s="2">
+      <c r="A69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" s="1">
         <v>238</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A70" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B70" s="2">
+      <c r="A70" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" s="1">
         <v>232</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A71" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B71" s="2">
+      <c r="A71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B71" s="1">
         <v>234</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A72" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B72" s="2">
+      <c r="A72" t="s">
+        <v>0</v>
+      </c>
+      <c r="B72" s="1">
         <v>219</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A73" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B73" s="2">
+      <c r="A73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B73" s="1">
         <v>236</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A74" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B74" s="2">
+      <c r="A74" t="s">
+        <v>0</v>
+      </c>
+      <c r="B74" s="1">
         <v>239</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A75" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B75" s="2">
+      <c r="A75" t="s">
+        <v>0</v>
+      </c>
+      <c r="B75" s="1">
         <v>215</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A76" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B76" s="2">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" s="1">
         <v>228</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A77" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B77" s="2">
+      <c r="A77" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" s="1">
         <v>240</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A78" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B78" s="2">
+      <c r="A78" t="s">
+        <v>0</v>
+      </c>
+      <c r="B78" s="1">
         <v>240</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A79" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B79" s="2">
+      <c r="A79" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" s="1">
         <v>237</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A80" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B80" s="2">
+      <c r="A80" t="s">
+        <v>0</v>
+      </c>
+      <c r="B80" s="1">
         <v>224</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A81" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B81" s="2">
+      <c r="A81" t="s">
+        <v>0</v>
+      </c>
+      <c r="B81" s="1">
         <v>229</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A82" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B82" s="2">
+      <c r="A82" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" s="1">
         <v>236</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A83" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B83" s="2">
+      <c r="A83" t="s">
+        <v>0</v>
+      </c>
+      <c r="B83" s="1">
         <v>238</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A84" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B84" s="2">
+      <c r="A84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" s="1">
         <v>245</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A85" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B85" s="2">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" s="1">
         <v>254</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A86" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B86" s="2">
+      <c r="A86" t="s">
+        <v>0</v>
+      </c>
+      <c r="B86" s="1">
         <v>228</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A87" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B87" s="2">
+      <c r="A87" t="s">
+        <v>0</v>
+      </c>
+      <c r="B87" s="1">
         <v>222</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A88" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B88" s="2">
+      <c r="A88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B88" s="1">
         <v>252</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A89" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B89" s="2">
+      <c r="A89" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="1">
         <v>214</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A90" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B90" s="2">
+      <c r="A90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B90" s="1">
         <v>220</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A91" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B91" s="2">
+      <c r="A91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B91" s="1">
         <v>234</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A92" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B92" s="2">
+      <c r="A92" t="s">
+        <v>0</v>
+      </c>
+      <c r="B92" s="1">
         <v>228</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A93" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B93" s="2">
+      <c r="A93" t="s">
+        <v>0</v>
+      </c>
+      <c r="B93" s="1">
         <v>222</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A94" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B94" s="2">
+      <c r="A94" t="s">
+        <v>0</v>
+      </c>
+      <c r="B94" s="1">
         <v>224</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A95" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B95" s="2">
+      <c r="A95" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" s="1">
         <v>236</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A96" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B96" s="2">
+      <c r="A96" t="s">
+        <v>0</v>
+      </c>
+      <c r="B96" s="1">
         <v>242</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A97" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B97" s="2">
+      <c r="A97" t="s">
+        <v>0</v>
+      </c>
+      <c r="B97" s="1">
         <v>228</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A98" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B98" s="2">
+      <c r="A98" t="s">
+        <v>0</v>
+      </c>
+      <c r="B98" s="1">
         <v>237</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A99" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B99" s="2">
+      <c r="A99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B99" s="1">
         <v>219</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A100" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B100" s="2">
+      <c r="A100" t="s">
+        <v>0</v>
+      </c>
+      <c r="B100" s="1">
         <v>218</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A101" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B101" s="2">
+      <c r="A101" t="s">
+        <v>0</v>
+      </c>
+      <c r="B101" s="1">
         <v>224</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A102" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B102" s="2">
+      <c r="A102" t="s">
+        <v>0</v>
+      </c>
+      <c r="B102" s="1">
         <v>220</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A103" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B103" s="2">
+      <c r="A103" t="s">
+        <v>0</v>
+      </c>
+      <c r="B103" s="1">
         <v>246</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A104" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B104" s="2">
+      <c r="A104" t="s">
+        <v>0</v>
+      </c>
+      <c r="B104" s="1">
         <v>240</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A105" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B105" s="2">
+      <c r="A105" t="s">
+        <v>0</v>
+      </c>
+      <c r="B105" s="1">
         <v>209</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A106" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B106" s="2">
+      <c r="A106" t="s">
+        <v>0</v>
+      </c>
+      <c r="B106" s="1">
         <v>234</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A107" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B107" s="2">
+      <c r="A107" t="s">
+        <v>0</v>
+      </c>
+      <c r="B107" s="1">
         <v>237</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A108" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B108" s="2">
+      <c r="A108" t="s">
+        <v>0</v>
+      </c>
+      <c r="B108" s="1">
         <v>201</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A109" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B109" s="2">
+      <c r="A109" t="s">
+        <v>0</v>
+      </c>
+      <c r="B109" s="1">
         <v>203</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A110" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B110" s="2">
+      <c r="A110" t="s">
+        <v>0</v>
+      </c>
+      <c r="B110" s="1">
         <v>257</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A111" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B111" s="2">
+      <c r="A111" t="s">
+        <v>0</v>
+      </c>
+      <c r="B111" s="1">
         <v>234</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A112" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B112" s="2">
+      <c r="A112" t="s">
+        <v>0</v>
+      </c>
+      <c r="B112" s="1">
         <v>218</v>
       </c>
     </row>

</xml_diff>